<commit_message>
Niveau 1-5 je Eintrag (KI-Vorschlag, editierbar), Spinnendiagramm je Kompetenzbereich, Excel-Spalte Niveau
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WVrt1ACeGcoC6nYYJLjo6w
</commit_message>
<xml_diff>
--- a/template/Skill-Diary-Vorlage.xlsx
+++ b/template/Skill-Diary-Vorlage.xlsx
@@ -147,9 +147,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Feedback" displayName="Feedback" ref="A1:N2" headerRowCount="1">
-  <autoFilter ref="A1:N2"/>
-  <tableColumns count="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Feedback" displayName="Feedback" ref="A1:O2" headerRowCount="1">
+  <autoFilter ref="A1:O2"/>
+  <tableColumns count="15">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Zeitstempel"/>
     <tableColumn id="3" name="Datum"/>
@@ -164,6 +164,7 @@
     <tableColumn id="12" name="Quelle"/>
     <tableColumn id="13" name="Gruppe"/>
     <tableColumn id="14" name="VideoLink"/>
+    <tableColumn id="15" name="Niveau"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showRowStripes="1"/>
 </table>
@@ -458,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3000"/>
+  <dimension ref="A1:O3000"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -475,6 +476,7 @@
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -548,6 +550,11 @@
           <t>VideoLink</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Niveau</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr"/>
@@ -564,6 +571,7 @@
       <c r="L2" s="1" t="inlineStr"/>
       <c r="M2" s="1" t="inlineStr"/>
       <c r="N2" s="1" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n"/>

</xml_diff>